<commit_message>
CI Reports [2026-06-25 16:05]: All — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report/Feature Reports/Dashboard.xlsx
+++ b/Test Execution Report/Feature Reports/Dashboard.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:O28"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="45.83203125" customWidth="1"/>
@@ -504,7 +504,7 @@
         <v>Automation (Playwright)</v>
       </c>
       <c r="M2" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="N2" t="str">
         <v/>
@@ -553,7 +553,7 @@
         <v>Automation (Playwright)</v>
       </c>
       <c r="M3" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="N3" t="str">
         <v>BUG-DASHBOARD-002</v>
@@ -602,7 +602,7 @@
         <v>Automation (Playwright)</v>
       </c>
       <c r="M4" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="N4" t="str">
         <v/>
@@ -651,7 +651,7 @@
         <v>Automation (Playwright)</v>
       </c>
       <c r="M5" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="N5" t="str">
         <v>BUG-DASHBOARD-004</v>
@@ -700,7 +700,7 @@
         <v>Automation (Playwright)</v>
       </c>
       <c r="M6" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="N6" t="str">
         <v>BUG-DASHBOARD-005</v>
@@ -749,7 +749,7 @@
         <v>Automation (Playwright)</v>
       </c>
       <c r="M7" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="N7" t="str">
         <v/>
@@ -798,7 +798,7 @@
         <v>Automation (Playwright)</v>
       </c>
       <c r="M8" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="N8" t="str">
         <v>BUG-DASHBOARD-007</v>
@@ -847,7 +847,7 @@
         <v>Automation (Playwright)</v>
       </c>
       <c r="M9" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="N9" t="str">
         <v/>
@@ -896,7 +896,7 @@
         <v>Automation (Playwright)</v>
       </c>
       <c r="M10" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="N10" t="str">
         <v/>
@@ -945,7 +945,7 @@
         <v>Automation (Playwright)</v>
       </c>
       <c r="M11" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="N11" t="str">
         <v/>
@@ -994,7 +994,7 @@
         <v>Automation (Playwright)</v>
       </c>
       <c r="M12" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="N12" t="str">
         <v>BUG-DASHBOARD-011</v>
@@ -1043,7 +1043,7 @@
         <v>Automation (Playwright)</v>
       </c>
       <c r="M13" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="N13" t="str">
         <v/>
@@ -1092,7 +1092,7 @@
         <v>Automation (Playwright)</v>
       </c>
       <c r="M14" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="N14" t="str">
         <v/>
@@ -1141,7 +1141,7 @@
         <v>Automation (Playwright)</v>
       </c>
       <c r="M15" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="N15" t="str">
         <v/>
@@ -1190,18 +1190,606 @@
         <v>Automation (Playwright)</v>
       </c>
       <c r="M16" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="N16" t="str">
         <v/>
       </c>
       <c r="O16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>TC-LOGIN-001</v>
+      </c>
+      <c r="B17" t="str">
+        <v>TC-LOGIN-001 | Login page loads with all UI elements</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D17" t="str">
+        <v>UI</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Username: sajith_xyz | Password: User@123</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K17" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="M17" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
+      <c r="O17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>TC-LOGIN-002</v>
+      </c>
+      <c r="B18" t="str">
+        <v>TC-LOGIN-002 | Valid credentials redirect to dashboard</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Username: sajith_xyz | Password: User@123</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J18" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K18" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="M18" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
+      <c r="O18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>TC-LOGIN-003</v>
+      </c>
+      <c r="B19" t="str">
+        <v>TC-LOGIN-003 | Login with Remember Me checked</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Username: sajith_xyz | Password: User@123</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K19" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="M19" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
+      <c r="O19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>TC-LOGIN-004</v>
+      </c>
+      <c r="B20" t="str">
+        <v>TC-LOGIN-004 | Invalid username shows error</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E20" t="str">
+        <v>High</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Username: sajith_xyz | Password: User@123</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K20" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L20" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="M20" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="N20" t="str">
+        <v/>
+      </c>
+      <c r="O20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>TC-LOGIN-005</v>
+      </c>
+      <c r="B21" t="str">
+        <v>TC-LOGIN-005 | Invalid password shows error</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E21" t="str">
+        <v>High</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Username: sajith_xyz | Password: User@123</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K21" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="M21" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="N21" t="str">
+        <v/>
+      </c>
+      <c r="O21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>TC-LOGIN-006</v>
+      </c>
+      <c r="B22" t="str">
+        <v>TC-LOGIN-006 | Empty username blocked</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="E22" t="str">
+        <v>High</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G22" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Username: sajith_xyz | Password: User@123</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K22" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L22" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="M22" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="N22" t="str">
+        <v/>
+      </c>
+      <c r="O22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>TC-LOGIN-007</v>
+      </c>
+      <c r="B23" t="str">
+        <v>TC-LOGIN-007 | Empty password blocked</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="E23" t="str">
+        <v>High</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G23" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Username: sajith_xyz | Password: User@123</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K23" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="M23" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="N23" t="str">
+        <v/>
+      </c>
+      <c r="O23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>TC-LOGIN-008</v>
+      </c>
+      <c r="B24" t="str">
+        <v>TC-LOGIN-008 | Both fields empty blocked</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="E24" t="str">
+        <v>High</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G24" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Username: sajith_xyz | Password: User@123</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K24" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L24" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="M24" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
+      <c r="O24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>TC-LOGIN-009</v>
+      </c>
+      <c r="B25" t="str">
+        <v>TC-LOGIN-009 | SQL injection rejected</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Security</v>
+      </c>
+      <c r="E25" t="str">
+        <v>High</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G25" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Username: sajith_xyz | Password: User@123</v>
+      </c>
+      <c r="I25" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J25" t="str">
+        <v>_x001b_[31mTest timeout of 30000ms exceeded._x001b_[39m</v>
+      </c>
+      <c r="K25" t="str">
+        <v>NOT RUN</v>
+      </c>
+      <c r="L25" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="M25" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="N25" t="str">
+        <v/>
+      </c>
+      <c r="O25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>TC-LOGIN-010</v>
+      </c>
+      <c r="B26" t="str">
+        <v>TC-LOGIN-010 | XSS payload rejected</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Security</v>
+      </c>
+      <c r="E26" t="str">
+        <v>High</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G26" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Username: sajith_xyz | Password: User@123</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K26" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L26" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="M26" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="N26" t="str">
+        <v/>
+      </c>
+      <c r="O26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
+        <v>TC-LOGIN-011</v>
+      </c>
+      <c r="B27" t="str">
+        <v>TC-LOGIN-011 | Max length username (256 chars) handled</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G27" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Username: sajith_xyz | Password: User@123</v>
+      </c>
+      <c r="I27" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J27" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K27" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L27" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="M27" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
+      <c r="O27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
+        <v>TC-LOGIN-012</v>
+      </c>
+      <c r="B28" t="str">
+        <v>TC-LOGIN-012 | Password field masks input</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D28" t="str">
+        <v>UI</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G28" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H28" t="str">
+        <v>Username: sajith_xyz | Password: User@123</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K28" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L28" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="M28" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="N28" t="str">
+        <v/>
+      </c>
+      <c r="O28" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O28"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1315,7 +1903,7 @@
         <v>New</v>
       </c>
       <c r="L2" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="M2" t="str">
         <v/>
@@ -1367,7 +1955,7 @@
         <v>New</v>
       </c>
       <c r="L3" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="M3" t="str">
         <v/>
@@ -1419,7 +2007,7 @@
         <v>New</v>
       </c>
       <c r="L4" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="M4" t="str">
         <v/>
@@ -1471,7 +2059,7 @@
         <v>New</v>
       </c>
       <c r="L5" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="M5" t="str">
         <v/>
@@ -1523,7 +2111,7 @@
         <v>New</v>
       </c>
       <c r="L6" t="str">
-        <v>24 Jun 2026</v>
+        <v>25 Jun 2026</v>
       </c>
       <c r="M6" t="str">
         <v/>

</xml_diff>